<commit_message>
feat: bo sung CLI test runner, Defect Tracking Log va Slide thuyet trinh
</commit_message>
<xml_diff>
--- a/Test_Case_Template.xlsx
+++ b/Test_Case_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function Test Cases" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security_Performanc Test Cases" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Test Cases ..." sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Tracking Log" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="d">'Function Test Cases'!$L$4</definedName>
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm\ d\,\ yyyy"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
@@ -119,8 +119,21 @@
       <color indexed="12"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -137,6 +150,12 @@
       <patternFill patternType="solid">
         <fgColor indexed="44"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -279,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -422,6 +441,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1110,9 +1144,6 @@
     <row r="3" customFormat="1" s="4"/>
     <row r="4" customFormat="1" s="4"/>
     <row r="5" customFormat="1" s="4"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
     <row r="9" ht="28" customFormat="1" customHeight="1" s="5">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
@@ -2237,7 +2268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="0.6640625" customWidth="1" min="1" max="1"/>
@@ -3259,24 +3290,13 @@
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="41" t="n"/>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3768,9 +3788,9 @@
   <mergeCells count="7">
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3790,7 +3810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="0.6640625" customWidth="1" min="1" max="1"/>
@@ -3804,383 +3824,372 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="44" t="inlineStr">
-        <is>
-          <t>Test Cases XYZ…</t>
-        </is>
-      </c>
-      <c r="B1" s="52" t="n"/>
-      <c r="C1" s="52" t="n"/>
-      <c r="D1" s="52" t="n"/>
-      <c r="E1" s="52" t="n"/>
-      <c r="F1" s="52" t="n"/>
-      <c r="G1" s="52" t="n"/>
-      <c r="H1" s="52" t="n"/>
+      <c r="A1" s="44" t="n"/>
+      <c r="B1" s="56" t="inlineStr">
+        <is>
+          <t>BẢNG THEO DÕI VÀ QUẢN LÝ LỖI (DEFECT TRACKING LOG)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>Each sheet should be used for a type of test such as Function Testing, User Interface Testing, Security Testing etc</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="H2" s="9">
-        <f>COUNTIF($H$9:$H$2001, "Passed")</f>
-        <v/>
-      </c>
+      <c r="B2" s="16" t="n"/>
+      <c r="G2" s="12" t="n"/>
+      <c r="H2" s="9" t="n"/>
     </row>
     <row r="3">
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="H3" s="9">
-        <f>COUNTIF($H$9:$H$2001, "Failed")</f>
-        <v/>
+      <c r="B3" s="57" t="inlineStr">
+        <is>
+          <t>Defect ID</t>
+        </is>
+      </c>
+      <c r="C3" s="57" t="inlineStr">
+        <is>
+          <t>Mô tả lỗi (Defect Description)</t>
+        </is>
+      </c>
+      <c r="D3" s="57" t="inlineStr">
+        <is>
+          <t>Mức độ (Severity)</t>
+        </is>
+      </c>
+      <c r="E3" s="57" t="inlineStr">
+        <is>
+          <t>Các bước tái hiện (Steps to Reproduce)</t>
+        </is>
+      </c>
+      <c r="F3" s="57" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế (Actual)</t>
+        </is>
+      </c>
+      <c r="G3" s="58" t="inlineStr">
+        <is>
+          <t>Kết quả kỳ vọng (Expected)</t>
+        </is>
+      </c>
+      <c r="H3" s="59" t="inlineStr">
+        <is>
+          <t>Trạng thái (Status)</t>
+        </is>
+      </c>
+      <c r="I3" s="57" t="inlineStr">
+        <is>
+          <t>Người sửa (Assignee)</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="13" t="n"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BUG_001</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Chấp nhận chỉ số công tơ là số âm (-50)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Nhập Cũ = -50, Mới = 100, bấm Tính</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Hệ thống vẫn tính ra 150 kWh</t>
+        </is>
+      </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="H4" s="9">
-        <f>COUNTIF($H$9:$H$2001, "Not Run")</f>
-        <v/>
+          <t>Phải chặn và báo lỗi 'Chỉ số cũ không được âm'</t>
+        </is>
+      </c>
+      <c r="H4" s="60" t="inlineStr">
+        <is>
+          <t>Closed (Đã sửa)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
       </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BUG_002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chấp nhận chỉ số thập phân (100.5 kWh)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Nhập Cũ = 100.5, Mới = 200, bấm Tính</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tiền điện ra số lẻ thập phân</t>
+        </is>
+      </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Not Completed</t>
-        </is>
-      </c>
-      <c r="H5" s="9">
-        <f>COUNTIF($H$9:$H$2001, "Not Completed")</f>
-        <v/>
+          <t>Phải chặn và yêu cầu số nguyên</t>
+        </is>
+      </c>
+      <c r="H5" s="60" t="inlineStr">
+        <is>
+          <t>Closed (Đã sửa)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
       </c>
     </row>
     <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BUG_003</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chỉ số mới &lt; Chỉ số cũ hệ thống tính tiền âm</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Nhập Cũ = 500, Mới = 300, bấm Tính</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Tiền ra số âm</t>
+        </is>
+      </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>Number of test cases</t>
-        </is>
-      </c>
-      <c r="H6" s="9">
-        <f>COUNTA(C9:C2000)</f>
-        <v/>
+          <t>Phải báo lỗi 'Chỉ số mới không được nhỏ hơn chỉ số cũ'</t>
+        </is>
+      </c>
+      <c r="H6" s="60" t="inlineStr">
+        <is>
+          <t>Closed (Đã sửa)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>BUG_004</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Test Case ID</t>
+          <t>Tiền thuế VAT không được làm tròn số nguyên đồng</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Test Case Description</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Test Procedures</t>
-        </is>
-      </c>
-      <c r="F7" s="50" t="n"/>
+          <t>Nhập Cũ = 0, Mới = 1 (VAT 8% = 158.72 đ)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Hiển thị 158.72 đ</t>
+        </is>
+      </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Test Case Expected Result</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Phải làm tròn Math.round thành 159 đ theo quy chuẩn tài chính</t>
+        </is>
+      </c>
+      <c r="H7" s="61" t="inlineStr">
+        <is>
+          <t>Closed (Đã sửa)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Developer</t>
         </is>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
-      <c r="B8" s="54" t="n"/>
-      <c r="C8" s="54" t="n"/>
-      <c r="D8" s="54" t="n"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BUG_005</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Trường hợp tiêu thụ 0 kWh bảng bậc thang bị lỗi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Steps to Perform</t>
+          <t>Nhập Cũ = 200, Mới = 200, bấm Tính</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Step Expected Result</t>
-        </is>
-      </c>
-      <c r="G8" s="54" t="n"/>
-      <c r="H8" s="54" t="n"/>
+          <t>Bảng bậc thang bị lỗi render</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Hiển thị 0 kWh và bảng các bậc dùng 0 kWh, tổng tiền 0 đ</t>
+        </is>
+      </c>
+      <c r="H8" s="62" t="inlineStr">
+        <is>
+          <t>Closed (Đã sửa)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
-      <c r="B9" s="40" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="C9" s="41" t="inlineStr">
-        <is>
-          <t>XYZ 001</t>
-        </is>
-      </c>
+      <c r="B9" s="40" t="n"/>
+      <c r="C9" s="41" t="n"/>
       <c r="D9" s="42" t="n"/>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Step description 1</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Expected result 1</t>
-        </is>
-      </c>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
       <c r="G9" s="43" t="n"/>
-      <c r="H9" s="41" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
+      <c r="H9" s="41" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="55" t="n"/>
-      <c r="C10" s="55" t="n"/>
-      <c r="D10" s="55" t="n"/>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Step description 2</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Expected result 2</t>
-        </is>
-      </c>
-      <c r="G10" s="55" t="n"/>
-      <c r="H10" s="55" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="55" t="n"/>
-      <c r="C11" s="54" t="n"/>
-      <c r="D11" s="54" t="n"/>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Step description n…</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Expected result n…</t>
-        </is>
-      </c>
-      <c r="G11" s="54" t="n"/>
-      <c r="H11" s="54" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="55" t="n"/>
-      <c r="C12" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 002</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Test 2</t>
-        </is>
-      </c>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="41" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="54" t="n"/>
-      <c r="C13" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 003</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Test 3</t>
-        </is>
-      </c>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="41" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 004</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Test 4</t>
-        </is>
-      </c>
+      <c r="B14" s="40" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="41" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="55" t="n"/>
-      <c r="C15" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 005</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Test 5</t>
-        </is>
-      </c>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="41" t="n"/>
     </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="B16" s="55" t="n"/>
-      <c r="C16" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 006</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Test 6</t>
-        </is>
-      </c>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="41" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="55" t="n"/>
-      <c r="C17" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 007</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Test 7</t>
-        </is>
-      </c>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="41" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="54" t="n"/>
-      <c r="C18" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 008</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Test 8</t>
-        </is>
-      </c>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="41" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="C19" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 009</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Test 9</t>
-        </is>
-      </c>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="41" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="55" t="n"/>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 010</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Test 10</t>
-        </is>
-      </c>
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="41" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="55" t="n"/>
-      <c r="C21" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 011</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Test 11</t>
-        </is>
-      </c>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="41" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="54" t="n"/>
-      <c r="C22" s="35" t="inlineStr">
-        <is>
-          <t>XYZ 012</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Test 12</t>
-        </is>
-      </c>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
@@ -4285,23 +4294,13 @@
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="41" t="n"/>
     </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="D9:D11"/>
-  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="H9:H33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>$G$2:$G$5</formula1>

</xml_diff>